<commit_message>
Add changes for solar panel temps
</commit_message>
<xml_diff>
--- a/genSpacecraft/DownlinkSpecFoxPlus-A.xlsx
+++ b/genSpacecraft/DownlinkSpecFoxPlus-A.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1379" uniqueCount="520">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1380" uniqueCount="522">
   <si>
     <t xml:space="preserve">//</t>
   </si>
@@ -713,6 +713,9 @@
     <t xml:space="preserve">plusXTemp</t>
   </si>
   <si>
+    <t xml:space="preserve">foxplus_solar_temps</t>
+  </si>
+  <si>
     <t xml:space="preserve">-X Panel Temp</t>
   </si>
   <si>
@@ -1023,6 +1026,9 @@
   </si>
   <si>
     <t xml:space="preserve">ModuGain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tlm_mod_reg1</t>
   </si>
   <si>
     <t xml:space="preserve">Modulator Register 1 - Gain</t>
@@ -5636,7 +5642,7 @@
       </c>
       <c r="F79" s="21"/>
       <c r="G79" s="21" t="s">
-        <v>76</v>
+        <v>230</v>
       </c>
       <c r="H79" s="20" t="s">
         <v>77</v>
@@ -5673,10 +5679,10 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B80" s="27" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C80" s="28" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D80" s="28" t="n">
         <v>8</v>
@@ -5686,7 +5692,7 @@
       </c>
       <c r="F80" s="21"/>
       <c r="G80" s="21" t="s">
-        <v>76</v>
+        <v>230</v>
       </c>
       <c r="H80" s="20" t="s">
         <v>77</v>
@@ -5723,10 +5729,10 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B81" s="27" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C81" s="28" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D81" s="28" t="n">
         <v>8</v>
@@ -5736,7 +5742,7 @@
       </c>
       <c r="F81" s="21"/>
       <c r="G81" s="21" t="s">
-        <v>76</v>
+        <v>230</v>
       </c>
       <c r="H81" s="20" t="s">
         <v>77</v>
@@ -5773,10 +5779,10 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B82" s="27" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C82" s="28" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D82" s="28" t="n">
         <v>8</v>
@@ -5786,7 +5792,7 @@
       </c>
       <c r="F82" s="21"/>
       <c r="G82" s="21" t="s">
-        <v>76</v>
+        <v>230</v>
       </c>
       <c r="H82" s="20" t="s">
         <v>77</v>
@@ -5823,10 +5829,10 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B83" s="27" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C83" s="28" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D83" s="28" t="n">
         <v>8</v>
@@ -5836,7 +5842,7 @@
       </c>
       <c r="F83" s="21"/>
       <c r="G83" s="21" t="s">
-        <v>76</v>
+        <v>230</v>
       </c>
       <c r="H83" s="20" t="s">
         <v>77</v>
@@ -5873,10 +5879,10 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B84" s="27" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C84" s="28" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D84" s="28" t="n">
         <v>16</v>
@@ -5931,7 +5937,7 @@
       <c r="G85" s="21"/>
       <c r="H85" s="21"/>
       <c r="I85" s="21" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J85" s="26" t="n">
         <f aca="false">J84+D84</f>
@@ -5969,7 +5975,7 @@
         <v>0</v>
       </c>
       <c r="B87" s="6" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C87" s="6"/>
       <c r="D87" s="6"/>
@@ -5981,7 +5987,7 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="1" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B88" s="27"/>
       <c r="C88" s="28"/>
@@ -5998,10 +6004,10 @@
     </row>
     <row r="89" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B89" s="27" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C89" s="28" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D89" s="28" t="n">
         <v>16</v>
@@ -6010,16 +6016,16 @@
         <v>26</v>
       </c>
       <c r="F89" s="21" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="G89" s="20" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="H89" s="20" t="s">
         <v>27</v>
       </c>
       <c r="I89" s="21" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="J89" s="26" t="n">
         <v>0</v>
@@ -6051,10 +6057,10 @@
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B90" s="27" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C90" s="27" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D90" s="28" t="n">
         <v>8</v>
@@ -6068,7 +6074,7 @@
       </c>
       <c r="H90" s="20"/>
       <c r="I90" s="28" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="J90" s="26" t="n">
         <f aca="false">J89+D89</f>
@@ -6107,7 +6113,7 @@
       <c r="C91" s="28"/>
       <c r="D91" s="28"/>
       <c r="E91" s="21" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F91" s="21"/>
       <c r="G91" s="21"/>
@@ -6123,10 +6129,10 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B92" s="27" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C92" s="27" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D92" s="28" t="n">
         <v>1</v>
@@ -6140,7 +6146,7 @@
       </c>
       <c r="H92" s="20"/>
       <c r="I92" s="28" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="J92" s="26" t="n">
         <f aca="false">J91+D91</f>
@@ -6173,10 +6179,10 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B93" s="27" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C93" s="28" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D93" s="28" t="n">
         <v>1</v>
@@ -6192,7 +6198,7 @@
         <v>27</v>
       </c>
       <c r="I93" s="21" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="J93" s="26" t="n">
         <f aca="false">J92+D92</f>
@@ -6225,10 +6231,10 @@
     </row>
     <row r="94" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B94" s="27" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C94" s="28" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D94" s="28" t="n">
         <v>1</v>
@@ -6244,7 +6250,7 @@
         <v>27</v>
       </c>
       <c r="I94" s="21" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="J94" s="26" t="n">
         <f aca="false">J93+D93</f>
@@ -6277,10 +6283,10 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B95" s="27" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C95" s="28" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D95" s="28" t="n">
         <v>1</v>
@@ -6296,7 +6302,7 @@
         <v>27</v>
       </c>
       <c r="I95" s="21" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="J95" s="26" t="n">
         <f aca="false">J94+D94</f>
@@ -6329,10 +6335,10 @@
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B96" s="27" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C96" s="28" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D96" s="28" t="n">
         <v>1</v>
@@ -6348,7 +6354,7 @@
         <v>27</v>
       </c>
       <c r="I96" s="21" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="J96" s="26" t="n">
         <f aca="false">J95+D95</f>
@@ -6381,10 +6387,10 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B97" s="27" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C97" s="28" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D97" s="28" t="n">
         <v>1</v>
@@ -6431,10 +6437,10 @@
     </row>
     <row r="98" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B98" s="29" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C98" s="28" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D98" s="28" t="n">
         <v>1</v>
@@ -6450,7 +6456,7 @@
         <v>27</v>
       </c>
       <c r="I98" s="21" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="J98" s="26" t="n">
         <f aca="false">J97+D97</f>
@@ -6483,10 +6489,10 @@
     </row>
     <row r="99" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B99" s="29" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C99" s="28" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D99" s="28" t="n">
         <v>1</v>
@@ -6496,13 +6502,13 @@
       </c>
       <c r="F99" s="21"/>
       <c r="G99" s="20" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="H99" s="20" t="s">
         <v>27</v>
       </c>
       <c r="I99" s="21" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="J99" s="26" t="n">
         <f aca="false">J98+D98</f>
@@ -6555,10 +6561,10 @@
     </row>
     <row r="101" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B101" s="27" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C101" s="28" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D101" s="28" t="n">
         <v>8</v>
@@ -6574,7 +6580,7 @@
         <v>27</v>
       </c>
       <c r="I101" s="21" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="J101" s="26" t="n">
         <f aca="false">J100+D100</f>
@@ -6607,10 +6613,10 @@
     </row>
     <row r="102" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B102" s="27" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C102" s="28" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D102" s="28" t="n">
         <v>8</v>
@@ -6626,7 +6632,7 @@
         <v>27</v>
       </c>
       <c r="I102" s="21" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="J102" s="26" t="n">
         <f aca="false">J101+D101</f>
@@ -6659,10 +6665,10 @@
     </row>
     <row r="103" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B103" s="27" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C103" s="28" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D103" s="28" t="n">
         <v>32</v>
@@ -6680,7 +6686,7 @@
         <v>27</v>
       </c>
       <c r="I103" s="21" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="J103" s="26" t="n">
         <f aca="false">J102+D102</f>
@@ -6713,10 +6719,10 @@
     </row>
     <row r="104" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B104" s="27" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C104" s="28" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D104" s="28" t="n">
         <v>8</v>
@@ -6732,7 +6738,7 @@
         <v>27</v>
       </c>
       <c r="I104" s="21" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="J104" s="26" t="n">
         <f aca="false">J103+D103</f>
@@ -6765,10 +6771,10 @@
     </row>
     <row r="105" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B105" s="27" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C105" s="28" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D105" s="28" t="n">
         <v>8</v>
@@ -6784,7 +6790,7 @@
         <v>27</v>
       </c>
       <c r="I105" s="21" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="J105" s="26" t="n">
         <f aca="false">J104+D104</f>
@@ -6817,10 +6823,10 @@
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B106" s="27" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C106" s="28" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D106" s="28" t="n">
         <v>16</v>
@@ -6832,13 +6838,13 @@
         <v>157</v>
       </c>
       <c r="G106" s="21" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="H106" s="20" t="s">
         <v>27</v>
       </c>
       <c r="I106" s="28" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="J106" s="26" t="n">
         <f aca="false">J105+D105</f>
@@ -6871,10 +6877,10 @@
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B107" s="27" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C107" s="28" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D107" s="28" t="n">
         <v>8</v>
@@ -6884,11 +6890,11 @@
       </c>
       <c r="F107" s="21"/>
       <c r="G107" s="20" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="H107" s="20"/>
       <c r="I107" s="28" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="J107" s="26" t="n">
         <f aca="false">J106+D106</f>
@@ -6921,10 +6927,10 @@
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B108" s="27" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C108" s="28" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D108" s="28" t="n">
         <v>1</v>
@@ -6934,7 +6940,7 @@
       </c>
       <c r="F108" s="21"/>
       <c r="G108" s="20" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="H108" s="20" t="s">
         <v>27</v>
@@ -6971,10 +6977,10 @@
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B109" s="27" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C109" s="28" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D109" s="28" t="n">
         <v>1</v>
@@ -6984,7 +6990,7 @@
       </c>
       <c r="F109" s="21"/>
       <c r="G109" s="20" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="H109" s="20" t="s">
         <v>27</v>
@@ -7021,10 +7027,10 @@
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B110" s="27" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C110" s="28" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D110" s="28" t="n">
         <v>1</v>
@@ -7034,7 +7040,7 @@
       </c>
       <c r="F110" s="21"/>
       <c r="G110" s="20" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="H110" s="20" t="s">
         <v>27</v>
@@ -7071,10 +7077,10 @@
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B111" s="27" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C111" s="28" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D111" s="28" t="n">
         <v>1</v>
@@ -7084,7 +7090,7 @@
       </c>
       <c r="F111" s="21"/>
       <c r="G111" s="20" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="H111" s="20" t="s">
         <v>27</v>
@@ -7121,10 +7127,10 @@
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B112" s="27" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C112" s="28" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D112" s="28" t="n">
         <v>1</v>
@@ -7134,7 +7140,7 @@
       </c>
       <c r="F112" s="21"/>
       <c r="G112" s="20" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="H112" s="20" t="s">
         <v>27</v>
@@ -7171,10 +7177,10 @@
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B113" s="27" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C113" s="28" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="D113" s="28" t="n">
         <v>1</v>
@@ -7184,7 +7190,7 @@
       </c>
       <c r="F113" s="21"/>
       <c r="G113" s="20" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="H113" s="20" t="s">
         <v>27</v>
@@ -7221,10 +7227,10 @@
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B114" s="27" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C114" s="28" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="D114" s="28" t="n">
         <v>1</v>
@@ -7234,11 +7240,11 @@
       </c>
       <c r="F114" s="21"/>
       <c r="G114" s="20" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="H114" s="20"/>
       <c r="I114" s="28" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="J114" s="26" t="n">
         <f aca="false">J113+D113</f>
@@ -7271,10 +7277,10 @@
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B115" s="27" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C115" s="28" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="D115" s="28" t="n">
         <v>1</v>
@@ -7284,7 +7290,7 @@
       </c>
       <c r="F115" s="21"/>
       <c r="G115" s="20" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="H115" s="20" t="s">
         <v>27</v>
@@ -7321,10 +7327,10 @@
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B116" s="27" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C116" s="28" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D116" s="28" t="n">
         <v>1</v>
@@ -7334,7 +7340,7 @@
       </c>
       <c r="F116" s="21"/>
       <c r="G116" s="20" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="H116" s="20" t="s">
         <v>27</v>
@@ -7371,10 +7377,10 @@
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B117" s="27" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C117" s="28" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D117" s="28" t="n">
         <v>1</v>
@@ -7384,7 +7390,7 @@
       </c>
       <c r="F117" s="21"/>
       <c r="G117" s="20" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="H117" s="20" t="s">
         <v>27</v>
@@ -7421,10 +7427,10 @@
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B118" s="27" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C118" s="28" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D118" s="28" t="n">
         <v>1</v>
@@ -7434,7 +7440,7 @@
       </c>
       <c r="F118" s="21"/>
       <c r="G118" s="20" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="H118" s="20" t="s">
         <v>27</v>
@@ -7471,10 +7477,10 @@
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B119" s="27" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C119" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D119" s="28" t="n">
         <v>1</v>
@@ -7484,7 +7490,7 @@
       </c>
       <c r="F119" s="21"/>
       <c r="G119" s="20" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="H119" s="20" t="s">
         <v>27</v>
@@ -7521,10 +7527,10 @@
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B120" s="27" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C120" s="28" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D120" s="28" t="n">
         <v>1</v>
@@ -7534,7 +7540,7 @@
       </c>
       <c r="F120" s="21"/>
       <c r="G120" s="20" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="H120" s="20" t="s">
         <v>27</v>
@@ -7571,10 +7577,10 @@
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B121" s="27" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C121" s="28" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D121" s="28" t="n">
         <v>1</v>
@@ -7584,7 +7590,7 @@
       </c>
       <c r="F121" s="21"/>
       <c r="G121" s="20" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="H121" s="20" t="s">
         <v>27</v>
@@ -7621,10 +7627,10 @@
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B122" s="27" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C122" s="28" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D122" s="28" t="n">
         <v>1</v>
@@ -7634,7 +7640,7 @@
       </c>
       <c r="F122" s="21"/>
       <c r="G122" s="20" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="H122" s="20" t="s">
         <v>27</v>
@@ -7671,10 +7677,10 @@
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B123" s="27" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C123" s="28" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="D123" s="28" t="n">
         <v>1</v>
@@ -7684,7 +7690,7 @@
       </c>
       <c r="F123" s="21"/>
       <c r="G123" s="20" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="H123" s="20" t="s">
         <v>27</v>
@@ -7721,10 +7727,10 @@
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B124" s="27" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C124" s="28" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D124" s="28" t="n">
         <v>8</v>
@@ -7740,7 +7746,7 @@
         <v>27</v>
       </c>
       <c r="I124" s="21" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="J124" s="26" t="n">
         <f aca="false">J123+D123</f>
@@ -7773,10 +7779,10 @@
     </row>
     <row r="125" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B125" s="27" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C125" s="28" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D125" s="28" t="n">
         <v>8</v>
@@ -7792,7 +7798,7 @@
         <v>27</v>
       </c>
       <c r="I125" s="21" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="J125" s="26" t="n">
         <f aca="false">J124+D124</f>
@@ -7825,10 +7831,10 @@
     </row>
     <row r="126" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B126" s="27" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C126" s="28" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D126" s="28" t="n">
         <v>8</v>
@@ -7837,14 +7843,14 @@
         <v>116</v>
       </c>
       <c r="F126" s="21"/>
-      <c r="G126" s="20" t="n">
-        <v>1</v>
+      <c r="G126" s="20" t="s">
+        <v>335</v>
       </c>
       <c r="H126" s="20" t="s">
         <v>27</v>
       </c>
       <c r="I126" s="21" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="J126" s="26" t="n">
         <f aca="false">J125+D125</f>
@@ -7877,10 +7883,10 @@
     </row>
     <row r="127" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B127" s="27" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="C127" s="28" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="D127" s="28" t="n">
         <v>8</v>
@@ -7896,7 +7902,7 @@
         <v>27</v>
       </c>
       <c r="I127" s="21" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="J127" s="26" t="n">
         <f aca="false">J126+D126</f>
@@ -7929,10 +7935,10 @@
     </row>
     <row r="128" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B128" s="27" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="C128" s="28" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="D128" s="28" t="n">
         <v>8</v>
@@ -7948,7 +7954,7 @@
         <v>27</v>
       </c>
       <c r="I128" s="21" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="J128" s="26" t="n">
         <f aca="false">J127+D127</f>
@@ -7981,10 +7987,10 @@
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B129" s="27" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="C129" s="28" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="D129" s="28" t="n">
         <v>16</v>
@@ -7994,7 +8000,7 @@
       </c>
       <c r="F129" s="21"/>
       <c r="G129" s="20" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="H129" s="20" t="s">
         <v>27</v>
@@ -8031,10 +8037,10 @@
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B130" s="27" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="C130" s="28" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="D130" s="28" t="n">
         <v>8</v>
@@ -8048,7 +8054,7 @@
       </c>
       <c r="H130" s="20"/>
       <c r="I130" s="28" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="J130" s="26" t="n">
         <f aca="false">J129+D129</f>
@@ -8103,10 +8109,10 @@
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B132" s="27" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="C132" s="27" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D132" s="28" t="n">
         <v>1</v>
@@ -8122,7 +8128,7 @@
         <v>27</v>
       </c>
       <c r="I132" s="21" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="J132" s="26" t="n">
         <f aca="false">J131+D131</f>
@@ -8152,10 +8158,10 @@
     </row>
     <row r="133" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B133" s="27" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="C133" s="28" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="D133" s="28" t="n">
         <v>1</v>
@@ -8171,7 +8177,7 @@
         <v>27</v>
       </c>
       <c r="I133" s="21" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="J133" s="26" t="n">
         <f aca="false">J132+D132</f>
@@ -8204,10 +8210,10 @@
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B134" s="27" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="C134" s="27" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="D134" s="28" t="n">
         <v>3</v>
@@ -8217,7 +8223,7 @@
       </c>
       <c r="F134" s="21"/>
       <c r="G134" s="21" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="H134" s="20" t="s">
         <v>27</v>
@@ -8254,10 +8260,10 @@
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B135" s="27" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="C135" s="28" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="D135" s="28" t="n">
         <v>1</v>
@@ -8304,10 +8310,10 @@
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B136" s="27" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="C136" s="28" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="D136" s="28" t="n">
         <v>1</v>
@@ -8323,7 +8329,7 @@
         <v>27</v>
       </c>
       <c r="I136" s="21" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="J136" s="26" t="n">
         <f aca="false">J135+D135</f>
@@ -8356,10 +8362,10 @@
     </row>
     <row r="137" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B137" s="27" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="C137" s="28" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="D137" s="28" t="n">
         <v>1</v>
@@ -8375,7 +8381,7 @@
         <v>27</v>
       </c>
       <c r="I137" s="21" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="J137" s="26" t="n">
         <f aca="false">J136+D136</f>
@@ -8428,10 +8434,10 @@
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B139" s="27" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="C139" s="27" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="D139" s="28" t="n">
         <v>8</v>
@@ -8445,7 +8451,7 @@
       </c>
       <c r="H139" s="20"/>
       <c r="I139" s="28" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="J139" s="26" t="n">
         <f aca="false">J138+D138</f>
@@ -8478,10 +8484,10 @@
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B140" s="27" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="C140" s="27" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="D140" s="28" t="n">
         <v>8</v>
@@ -8495,7 +8501,7 @@
       </c>
       <c r="H140" s="20"/>
       <c r="I140" s="28" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="J140" s="26" t="n">
         <f aca="false">J139+D139</f>
@@ -8528,10 +8534,10 @@
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B141" s="27" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="C141" s="27" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="D141" s="28" t="n">
         <v>32</v>
@@ -8545,7 +8551,7 @@
       </c>
       <c r="H141" s="20"/>
       <c r="I141" s="28" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="J141" s="26" t="n">
         <f aca="false">J140+D140</f>
@@ -8588,7 +8594,7 @@
       <c r="G142" s="32"/>
       <c r="H142" s="31"/>
       <c r="I142" s="32" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="J142" s="26" t="n">
         <f aca="false">J141+D141</f>
@@ -8621,7 +8627,7 @@
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="1" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B145" s="27"/>
       <c r="C145" s="28"/>
@@ -8641,7 +8647,7 @@
         <v>57</v>
       </c>
       <c r="C146" s="28" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="D146" s="28" t="n">
         <v>32</v>
@@ -8699,7 +8705,7 @@
       <c r="G147" s="32"/>
       <c r="H147" s="31"/>
       <c r="I147" s="32" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="J147" s="26" t="n">
         <f aca="false">J146+D146</f>
@@ -8736,31 +8742,31 @@
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="1" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B150" s="27" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="C150" s="28" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="D150" s="25" t="n">
         <v>32</v>
       </c>
       <c r="E150" s="34" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="F150" s="21"/>
       <c r="G150" s="35" t="n">
         <v>0</v>
       </c>
       <c r="H150" s="3" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="I150" s="26" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="J150" s="26" t="n">
         <f aca="false">J85</f>
@@ -8793,10 +8799,10 @@
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B151" s="27" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="C151" s="28" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="D151" s="25" t="n">
         <v>16</v>
@@ -8806,11 +8812,11 @@
       </c>
       <c r="F151" s="21"/>
       <c r="G151" s="21" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="H151" s="35"/>
       <c r="I151" s="26" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="J151" s="26" t="n">
         <f aca="false">J150+D150</f>
@@ -8829,7 +8835,7 @@
         <v>18</v>
       </c>
       <c r="N151" s="1" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="O151" s="3" t="n">
         <v>5</v>
@@ -8843,26 +8849,26 @@
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B152" s="27" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="C152" s="28" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="D152" s="25" t="n">
         <v>8</v>
       </c>
       <c r="E152" s="34" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="F152" s="21"/>
       <c r="G152" s="21" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="H152" s="20" t="s">
         <v>27</v>
       </c>
       <c r="I152" s="26" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="J152" s="26" t="n">
         <f aca="false">J151+D151</f>
@@ -8881,7 +8887,7 @@
         <v>18.5</v>
       </c>
       <c r="N152" s="1" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="O152" s="3" t="n">
         <v>5</v>
@@ -8895,10 +8901,10 @@
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B153" s="27" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="C153" s="28" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="D153" s="25" t="n">
         <v>8</v>
@@ -8912,7 +8918,7 @@
         <v>27</v>
       </c>
       <c r="I153" s="26" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="J153" s="26" t="n">
         <f aca="false">J152+D152</f>
@@ -8954,7 +8960,7 @@
       <c r="G154" s="32"/>
       <c r="H154" s="31"/>
       <c r="I154" s="32" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="J154" s="26" t="n">
         <f aca="false">J153+D153</f>
@@ -8975,15 +8981,15 @@
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="1" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B158" s="27" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="C158" s="28" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="D158" s="25" t="n">
         <v>32</v>
@@ -8995,7 +9001,7 @@
       </c>
       <c r="H158" s="35"/>
       <c r="I158" s="26" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="J158" s="26" t="n">
         <f aca="false">J85</f>
@@ -9028,10 +9034,10 @@
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B159" s="27" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="C159" s="28" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="D159" s="25" t="n">
         <v>16</v>
@@ -9041,10 +9047,10 @@
       </c>
       <c r="F159" s="21"/>
       <c r="G159" s="21" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="I159" s="26" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="J159" s="26" t="n">
         <f aca="false">J158+D158</f>
@@ -9063,7 +9069,7 @@
         <v>18</v>
       </c>
       <c r="N159" s="1" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="O159" s="3" t="n">
         <v>5</v>
@@ -9077,10 +9083,10 @@
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B160" s="27" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="C160" s="28" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="D160" s="25" t="n">
         <v>16</v>
@@ -9088,10 +9094,10 @@
       <c r="E160" s="34"/>
       <c r="F160" s="21"/>
       <c r="G160" s="21" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="I160" s="26" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="J160" s="26" t="n">
         <f aca="false">J159+D159</f>
@@ -9110,7 +9116,7 @@
         <v>18.5</v>
       </c>
       <c r="N160" s="1" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="O160" s="3" t="n">
         <v>5</v>
@@ -9124,10 +9130,10 @@
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B161" s="1" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="C161" s="28" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="D161" s="25" t="n">
         <v>32</v>
@@ -9138,7 +9144,7 @@
         <v>0</v>
       </c>
       <c r="I161" s="26" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="J161" s="26" t="n">
         <f aca="false">J160+D160</f>
@@ -9171,26 +9177,26 @@
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B162" s="27" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="C162" s="28" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="D162" s="25" t="n">
         <v>8</v>
       </c>
       <c r="E162" s="34" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="F162" s="21"/>
       <c r="G162" s="21" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="H162" s="20" t="s">
         <v>27</v>
       </c>
       <c r="I162" s="26" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="J162" s="26" t="n">
         <f aca="false">J161+D161</f>
@@ -9209,7 +9215,7 @@
         <v>20</v>
       </c>
       <c r="N162" s="1" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="O162" s="3" t="n">
         <v>5</v>
@@ -9223,10 +9229,10 @@
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B163" s="27" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="C163" s="28" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="D163" s="25" t="n">
         <v>24</v>
@@ -9283,7 +9289,7 @@
       <c r="G164" s="32"/>
       <c r="H164" s="31"/>
       <c r="I164" s="32" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="J164" s="26" t="n">
         <f aca="false">J163+D163</f>
@@ -9309,15 +9315,15 @@
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="1" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B169" s="27" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="C169" s="28" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="D169" s="25" t="n">
         <v>32</v>
@@ -9330,10 +9336,10 @@
         <v>1</v>
       </c>
       <c r="H169" s="37" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="I169" s="26" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="J169" s="26" t="n">
         <f aca="false">J142</f>
@@ -9366,10 +9372,10 @@
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B170" s="27" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="C170" s="28" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="D170" s="25" t="n">
         <v>16</v>
@@ -9379,13 +9385,13 @@
       </c>
       <c r="F170" s="21"/>
       <c r="G170" s="21" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="H170" s="37" t="s">
         <v>27</v>
       </c>
       <c r="I170" s="26" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="J170" s="26" t="n">
         <f aca="false">J169+D169</f>
@@ -9404,7 +9410,7 @@
         <v>9</v>
       </c>
       <c r="N170" s="1" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="O170" s="3" t="n">
         <v>5</v>
@@ -9418,10 +9424,10 @@
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B171" s="27" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="C171" s="28" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="D171" s="25" t="n">
         <v>1</v>
@@ -9431,13 +9437,13 @@
       </c>
       <c r="F171" s="21"/>
       <c r="G171" s="37" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="H171" s="20" t="s">
         <v>27</v>
       </c>
       <c r="I171" s="26" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="J171" s="26" t="n">
         <f aca="false">J170+D170</f>
@@ -9456,7 +9462,7 @@
         <v>9.5</v>
       </c>
       <c r="N171" s="4" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="O171" s="22" t="n">
         <v>5</v>
@@ -9646,7 +9652,7 @@
         <v>55</v>
       </c>
       <c r="C176" s="20" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="D176" s="20" t="n">
         <v>12</v>
@@ -9714,7 +9720,7 @@
       </c>
       <c r="B178" s="27"/>
       <c r="I178" s="1" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J178" s="26" t="n">
         <f aca="false">J176+D176</f>
@@ -9735,7 +9741,7 @@
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="38" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B179" s="10"/>
       <c r="C179" s="39"/>
@@ -9801,10 +9807,10 @@
     </row>
     <row r="181" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B181" s="27" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="C181" s="20" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D181" s="20" t="n">
         <v>5216</v>
@@ -9822,7 +9828,7 @@
         <v>27</v>
       </c>
       <c r="I181" s="21" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="J181" s="4" t="n">
         <v>0</v>
@@ -9854,10 +9860,10 @@
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B182" s="27" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="C182" s="20" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D182" s="20" t="n">
         <v>7</v>
@@ -9906,10 +9912,10 @@
     </row>
     <row r="183" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B183" s="27" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="C183" s="20" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="D183" s="20" t="n">
         <v>1</v>
@@ -9923,7 +9929,7 @@
       </c>
       <c r="H183" s="20"/>
       <c r="I183" s="21" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="J183" s="4" t="n">
         <f aca="false">J182+D182</f>
@@ -9942,7 +9948,7 @@
         <v>163.21875</v>
       </c>
       <c r="N183" s="1" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="O183" s="3" t="n">
         <v>1</v>
@@ -9959,7 +9965,7 @@
         <v>59</v>
       </c>
       <c r="I184" s="1" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J184" s="4" t="n">
         <f aca="false">J183+D183</f>
@@ -9987,7 +9993,7 @@
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="40" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B186" s="10"/>
       <c r="C186" s="39"/>
@@ -10053,10 +10059,10 @@
     </row>
     <row r="188" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B188" s="27" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="C188" s="20" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D188" s="20" t="n">
         <v>664</v>
@@ -10074,7 +10080,7 @@
         <v>27</v>
       </c>
       <c r="I188" s="21" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="J188" s="4" t="n">
         <v>0</v>
@@ -10106,10 +10112,10 @@
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B189" s="27" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="C189" s="20" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="D189" s="20" t="n">
         <v>7</v>
@@ -10158,10 +10164,10 @@
     </row>
     <row r="190" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B190" s="27" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="C190" s="20" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="D190" s="20" t="n">
         <v>1</v>
@@ -10175,7 +10181,7 @@
       </c>
       <c r="H190" s="20"/>
       <c r="I190" s="21" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="J190" s="4" t="n">
         <f aca="false">J189+D189</f>
@@ -10194,7 +10200,7 @@
         <v>20.96875</v>
       </c>
       <c r="N190" s="1" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="O190" s="3" t="n">
         <v>1</v>
@@ -10211,7 +10217,7 @@
         <v>59</v>
       </c>
       <c r="I191" s="1" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J191" s="4" t="n">
         <f aca="false">J190+D190</f>
@@ -10232,7 +10238,7 @@
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A195" s="40" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B195" s="10"/>
       <c r="C195" s="39"/>
@@ -10298,10 +10304,10 @@
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B197" s="27" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="C197" s="28" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="D197" s="25" t="n">
         <v>32</v>
@@ -10314,10 +10320,10 @@
         <v>1</v>
       </c>
       <c r="H197" s="37" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="I197" s="26" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="J197" s="4" t="n">
         <f aca="false">J191</f>
@@ -10350,10 +10356,10 @@
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B198" s="27" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="C198" s="28" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="D198" s="25" t="n">
         <v>16</v>
@@ -10365,13 +10371,13 @@
         <v>157</v>
       </c>
       <c r="G198" s="21" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="H198" s="37" t="s">
         <v>27</v>
       </c>
       <c r="I198" s="26" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="J198" s="4" t="n">
         <f aca="false">J197+D197</f>
@@ -10390,7 +10396,7 @@
         <v>22</v>
       </c>
       <c r="N198" s="1" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="O198" s="3" t="n">
         <v>2</v>
@@ -10404,10 +10410,10 @@
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B199" s="27" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="C199" s="28" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="D199" s="25" t="n">
         <v>8</v>
@@ -10415,13 +10421,13 @@
       <c r="E199" s="34"/>
       <c r="F199" s="21"/>
       <c r="G199" s="37" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="H199" s="37" t="s">
         <v>27</v>
       </c>
       <c r="I199" s="26" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="J199" s="4" t="n">
         <f aca="false">J198+D198</f>
@@ -10440,7 +10446,7 @@
         <v>22.5</v>
       </c>
       <c r="N199" s="4" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="O199" s="22" t="n">
         <v>2</v>
@@ -10457,7 +10463,7 @@
         <v>28</v>
       </c>
       <c r="C200" s="28" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="D200" s="25" t="n">
         <v>8</v>
@@ -10471,7 +10477,7 @@
         <v>27</v>
       </c>
       <c r="I200" s="26" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="J200" s="4" t="n">
         <f aca="false">J199+D199</f>
@@ -10507,7 +10513,7 @@
         <v>59</v>
       </c>
       <c r="I201" s="1" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J201" s="4" t="n">
         <f aca="false">J200+D200</f>
@@ -10540,7 +10546,7 @@
     </row>
     <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A203" s="40" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
     </row>
     <row r="204" s="13" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10598,10 +10604,10 @@
     </row>
     <row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B205" s="41" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C205" s="34" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="D205" s="34" t="n">
         <v>32</v>
@@ -10611,13 +10617,13 @@
       </c>
       <c r="F205" s="34"/>
       <c r="G205" s="34" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="H205" s="34" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="I205" s="34" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="J205" s="42" t="n">
         <v>0</v>
@@ -10635,7 +10641,7 @@
         <v>0</v>
       </c>
       <c r="N205" s="1" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="O205" s="3" t="n">
         <v>1</v>
@@ -10649,10 +10655,10 @@
     </row>
     <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B206" s="41" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="C206" s="34" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="D206" s="34" t="n">
         <v>32</v>
@@ -10662,13 +10668,13 @@
       </c>
       <c r="F206" s="34"/>
       <c r="G206" s="34" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="H206" s="34" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="I206" s="34" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="J206" s="42" t="n">
         <f aca="false">J205+D205</f>
@@ -10687,7 +10693,7 @@
         <v>1</v>
       </c>
       <c r="N206" s="1" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="O206" s="3" t="n">
         <v>1</v>
@@ -10701,7 +10707,7 @@
     </row>
     <row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A207" s="1" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B207" s="41"/>
       <c r="C207" s="34"/>
@@ -10718,10 +10724,10 @@
     </row>
     <row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B208" s="41" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="C208" s="34" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="D208" s="34" t="n">
         <v>1</v>
@@ -10731,13 +10737,13 @@
       </c>
       <c r="F208" s="34"/>
       <c r="G208" s="34" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="H208" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I208" s="34" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J208" s="42" t="n">
         <f aca="false">J206+D206</f>
@@ -10756,7 +10762,7 @@
         <v>2</v>
       </c>
       <c r="N208" s="1" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="O208" s="3" t="n">
         <v>1</v>
@@ -10770,10 +10776,10 @@
     </row>
     <row r="209" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B209" s="41" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="C209" s="34" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="D209" s="34" t="n">
         <v>5</v>
@@ -10783,11 +10789,11 @@
       </c>
       <c r="F209" s="34"/>
       <c r="G209" s="34" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="H209" s="34"/>
       <c r="I209" s="34" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="J209" s="42" t="n">
         <f aca="false">J208+D208</f>
@@ -10806,7 +10812,7 @@
         <v>2.03125</v>
       </c>
       <c r="N209" s="1" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="O209" s="3" t="n">
         <v>1</v>
@@ -10820,10 +10826,10 @@
     </row>
     <row r="210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B210" s="41" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="C210" s="34" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="D210" s="34" t="n">
         <v>4</v>
@@ -10833,13 +10839,13 @@
       </c>
       <c r="F210" s="34"/>
       <c r="G210" s="34" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="H210" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I210" s="34" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J210" s="42" t="n">
         <f aca="false">J209+D209</f>
@@ -10858,7 +10864,7 @@
         <v>2.1875</v>
       </c>
       <c r="N210" s="1" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="O210" s="3" t="n">
         <v>1</v>
@@ -10872,10 +10878,10 @@
     </row>
     <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B211" s="41" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="C211" s="34" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="D211" s="34" t="n">
         <v>5</v>
@@ -10885,13 +10891,13 @@
       </c>
       <c r="F211" s="34"/>
       <c r="G211" s="34" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="H211" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I211" s="34" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J211" s="42" t="n">
         <f aca="false">J210+D210</f>
@@ -10910,7 +10916,7 @@
         <v>2.3125</v>
       </c>
       <c r="N211" s="1" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="O211" s="3" t="n">
         <v>1</v>
@@ -10924,10 +10930,10 @@
     </row>
     <row r="212" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B212" s="41" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="C212" s="34" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="D212" s="34" t="n">
         <v>6</v>
@@ -10937,13 +10943,13 @@
       </c>
       <c r="F212" s="34"/>
       <c r="G212" s="34" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="H212" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I212" s="34" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J212" s="42" t="n">
         <f aca="false">J211+D211</f>
@@ -10962,7 +10968,7 @@
         <v>2.46875</v>
       </c>
       <c r="N212" s="1" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="O212" s="3" t="n">
         <v>1</v>
@@ -10976,10 +10982,10 @@
     </row>
     <row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B213" s="41" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="C213" s="34" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="D213" s="34" t="n">
         <v>6</v>
@@ -10989,13 +10995,13 @@
       </c>
       <c r="F213" s="34"/>
       <c r="G213" s="34" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="H213" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I213" s="34" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J213" s="42" t="n">
         <f aca="false">J212+D212</f>
@@ -11014,7 +11020,7 @@
         <v>2.65625</v>
       </c>
       <c r="N213" s="1" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="O213" s="3" t="n">
         <v>1</v>
@@ -11028,10 +11034,10 @@
     </row>
     <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B214" s="41" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="C214" s="34" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="D214" s="34" t="n">
         <v>5</v>
@@ -11041,13 +11047,13 @@
       </c>
       <c r="F214" s="34"/>
       <c r="G214" s="34" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="H214" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I214" s="34" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J214" s="42" t="n">
         <f aca="false">J213+D213</f>
@@ -11066,7 +11072,7 @@
         <v>2.84375</v>
       </c>
       <c r="N214" s="1" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="O214" s="3" t="n">
         <v>1</v>
@@ -11080,7 +11086,7 @@
     </row>
     <row r="215" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A215" s="1" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B215" s="41"/>
       <c r="C215" s="34"/>
@@ -11097,10 +11103,10 @@
     </row>
     <row r="216" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B216" s="41" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="C216" s="34" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="D216" s="34" t="n">
         <v>8</v>
@@ -11116,7 +11122,7 @@
         <v>71</v>
       </c>
       <c r="I216" s="34" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J216" s="42" t="n">
         <f aca="false">J214+D214</f>
@@ -11135,7 +11141,7 @@
         <v>3</v>
       </c>
       <c r="N216" s="1" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="O216" s="3" t="n">
         <v>1</v>
@@ -11149,10 +11155,10 @@
     </row>
     <row r="217" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B217" s="41" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="C217" s="34" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="D217" s="34" t="n">
         <v>8</v>
@@ -11168,7 +11174,7 @@
         <v>71</v>
       </c>
       <c r="I217" s="34" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J217" s="42" t="n">
         <f aca="false">J216+D216</f>
@@ -11187,7 +11193,7 @@
         <v>3.25</v>
       </c>
       <c r="N217" s="1" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="O217" s="3" t="n">
         <v>1</v>
@@ -11201,10 +11207,10 @@
     </row>
     <row r="218" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B218" s="41" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="C218" s="34" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="D218" s="34" t="n">
         <v>8</v>
@@ -11220,7 +11226,7 @@
         <v>27</v>
       </c>
       <c r="I218" s="34" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J218" s="42" t="n">
         <f aca="false">J217+D217</f>
@@ -11253,10 +11259,10 @@
     </row>
     <row r="219" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B219" s="41" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="C219" s="34" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="D219" s="34" t="n">
         <v>8</v>
@@ -11266,13 +11272,13 @@
       </c>
       <c r="F219" s="34"/>
       <c r="G219" s="34" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="H219" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I219" s="34" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J219" s="42" t="n">
         <f aca="false">J218+D218</f>
@@ -11291,7 +11297,7 @@
         <v>3.75</v>
       </c>
       <c r="N219" s="1" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="O219" s="3" t="n">
         <v>2</v>
@@ -11314,7 +11320,7 @@
       <c r="G220" s="34"/>
       <c r="H220" s="34"/>
       <c r="I220" s="34" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J220" s="42" t="n">
         <f aca="false">J219+D219</f>
@@ -11335,7 +11341,7 @@
     </row>
     <row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A221" s="40" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="F221" s="34"/>
       <c r="G221" s="34"/>
@@ -11419,10 +11425,10 @@
     </row>
     <row r="224" s="45" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B224" s="19" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="C224" s="43" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="D224" s="1" t="n">
         <v>5</v>
@@ -11438,7 +11444,7 @@
         <v>27</v>
       </c>
       <c r="I224" s="34" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J224" s="42" t="n">
         <f aca="false">J220</f>
@@ -11471,10 +11477,10 @@
     </row>
     <row r="225" s="45" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B225" s="19" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="C225" s="43" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="D225" s="1" t="n">
         <v>1</v>
@@ -11484,13 +11490,13 @@
       </c>
       <c r="F225" s="44"/>
       <c r="G225" s="34" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="H225" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I225" s="34" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J225" s="42" t="n">
         <f aca="false">J224+D224</f>
@@ -11509,7 +11515,7 @@
         <v>4.15625</v>
       </c>
       <c r="N225" s="1" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="O225" s="3" t="n">
         <v>1</v>
@@ -11523,10 +11529,10 @@
     </row>
     <row r="226" s="45" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B226" s="19" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="C226" s="43" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="D226" s="1" t="n">
         <v>1</v>
@@ -11536,13 +11542,13 @@
       </c>
       <c r="F226" s="44"/>
       <c r="G226" s="34" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="H226" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I226" s="34" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J226" s="42" t="n">
         <f aca="false">J225+D225</f>
@@ -11561,7 +11567,7 @@
         <v>4.1875</v>
       </c>
       <c r="N226" s="1" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="O226" s="3" t="n">
         <v>2</v>
@@ -11575,10 +11581,10 @@
     </row>
     <row r="227" s="45" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B227" s="19" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="C227" s="43" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="D227" s="1" t="n">
         <v>3</v>
@@ -11588,13 +11594,13 @@
       </c>
       <c r="F227" s="44"/>
       <c r="G227" s="34" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="H227" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I227" s="34" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J227" s="42" t="n">
         <f aca="false">J226+D226</f>
@@ -11613,7 +11619,7 @@
         <v>4.21875</v>
       </c>
       <c r="N227" s="1" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="O227" s="3" t="n">
         <v>2</v>
@@ -11627,10 +11633,10 @@
     </row>
     <row r="228" s="45" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B228" s="19" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="C228" s="43" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="D228" s="1" t="n">
         <v>4</v>
@@ -11640,13 +11646,13 @@
       </c>
       <c r="F228" s="44"/>
       <c r="G228" s="34" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="H228" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I228" s="34" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J228" s="42" t="n">
         <f aca="false">J227+D227</f>
@@ -11665,7 +11671,7 @@
         <v>4.3125</v>
       </c>
       <c r="N228" s="1" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="O228" s="3" t="n">
         <v>2</v>
@@ -11679,10 +11685,10 @@
     </row>
     <row r="229" s="45" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B229" s="19" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="C229" s="43" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="D229" s="1" t="n">
         <v>4</v>
@@ -11692,13 +11698,13 @@
       </c>
       <c r="F229" s="44"/>
       <c r="G229" s="34" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="H229" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I229" s="34" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J229" s="42" t="n">
         <f aca="false">J228+D228</f>
@@ -11717,7 +11723,7 @@
         <v>4.4375</v>
       </c>
       <c r="N229" s="1" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="O229" s="3" t="n">
         <v>2</v>
@@ -11731,10 +11737,10 @@
     </row>
     <row r="230" s="45" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B230" s="19" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="C230" s="43" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="D230" s="1" t="n">
         <v>5</v>
@@ -11744,13 +11750,13 @@
       </c>
       <c r="F230" s="44"/>
       <c r="G230" s="34" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="H230" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I230" s="34" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J230" s="42" t="n">
         <f aca="false">J229+D229</f>
@@ -11769,7 +11775,7 @@
         <v>4.5625</v>
       </c>
       <c r="N230" s="1" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="O230" s="3" t="n">
         <v>2</v>
@@ -11783,10 +11789,10 @@
     </row>
     <row r="231" s="45" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B231" s="19" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="C231" s="43" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="D231" s="1" t="n">
         <v>9</v>
@@ -11796,13 +11802,13 @@
       </c>
       <c r="F231" s="44"/>
       <c r="G231" s="34" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="H231" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I231" s="34" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J231" s="42" t="n">
         <f aca="false">J230+D230</f>
@@ -11821,7 +11827,7 @@
         <v>4.71875</v>
       </c>
       <c r="N231" s="1" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="O231" s="3" t="n">
         <v>2</v>
@@ -11854,10 +11860,10 @@
     </row>
     <row r="233" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B233" s="45" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="C233" s="3" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="D233" s="1" t="n">
         <v>8</v>
@@ -11867,13 +11873,13 @@
       </c>
       <c r="F233" s="34"/>
       <c r="G233" s="34" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="H233" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I233" s="34" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J233" s="42" t="n">
         <f aca="false">J231+D231</f>
@@ -11892,7 +11898,7 @@
         <v>5</v>
       </c>
       <c r="N233" s="1" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="O233" s="3" t="n">
         <v>3</v>
@@ -11906,10 +11912,10 @@
     </row>
     <row r="234" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B234" s="45" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="C234" s="3" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="D234" s="1" t="n">
         <v>8</v>
@@ -11919,13 +11925,13 @@
       </c>
       <c r="F234" s="34"/>
       <c r="G234" s="34" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="H234" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I234" s="34" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J234" s="42" t="n">
         <f aca="false">J233+D233</f>
@@ -11944,7 +11950,7 @@
         <v>5.25</v>
       </c>
       <c r="N234" s="1" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="O234" s="3" t="n">
         <v>3</v>
@@ -11958,10 +11964,10 @@
     </row>
     <row r="235" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B235" s="45" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="C235" s="3" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="D235" s="1" t="n">
         <v>8</v>
@@ -11971,13 +11977,13 @@
       </c>
       <c r="F235" s="34"/>
       <c r="G235" s="34" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="H235" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I235" s="34" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J235" s="42" t="n">
         <f aca="false">J234+D234</f>
@@ -11996,7 +12002,7 @@
         <v>5.5</v>
       </c>
       <c r="N235" s="1" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="O235" s="3" t="n">
         <v>3</v>
@@ -12010,10 +12016,10 @@
     </row>
     <row r="236" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B236" s="45" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="C236" s="3" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="D236" s="1" t="n">
         <v>8</v>
@@ -12023,13 +12029,13 @@
       </c>
       <c r="F236" s="34"/>
       <c r="G236" s="34" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="H236" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I236" s="34" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J236" s="42" t="n">
         <f aca="false">J235+D235</f>
@@ -12048,7 +12054,7 @@
         <v>5.75</v>
       </c>
       <c r="N236" s="1" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="O236" s="3" t="n">
         <v>3</v>
@@ -12062,10 +12068,10 @@
     </row>
     <row r="237" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B237" s="45" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="C237" s="3" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="D237" s="1" t="n">
         <v>8</v>
@@ -12075,13 +12081,13 @@
       </c>
       <c r="F237" s="34"/>
       <c r="G237" s="34" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="H237" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I237" s="34" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J237" s="42" t="n">
         <f aca="false">J236+D236</f>
@@ -12100,7 +12106,7 @@
         <v>6</v>
       </c>
       <c r="N237" s="1" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="O237" s="3" t="n">
         <v>3</v>
@@ -12114,10 +12120,10 @@
     </row>
     <row r="238" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B238" s="45" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="C238" s="3" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="D238" s="1" t="n">
         <v>8</v>
@@ -12127,13 +12133,13 @@
       </c>
       <c r="F238" s="34"/>
       <c r="G238" s="34" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="H238" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I238" s="34" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J238" s="42" t="n">
         <f aca="false">J237+D237</f>
@@ -12152,7 +12158,7 @@
         <v>6.25</v>
       </c>
       <c r="N238" s="1" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="O238" s="3" t="n">
         <v>3</v>
@@ -12166,10 +12172,10 @@
     </row>
     <row r="239" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B239" s="45" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="C239" s="3" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="D239" s="1" t="n">
         <v>8</v>
@@ -12179,13 +12185,13 @@
       </c>
       <c r="F239" s="34"/>
       <c r="G239" s="34" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="H239" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I239" s="34" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J239" s="42" t="n">
         <f aca="false">J238+D238</f>
@@ -12204,7 +12210,7 @@
         <v>6.5</v>
       </c>
       <c r="N239" s="1" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="O239" s="3" t="n">
         <v>3</v>
@@ -12218,10 +12224,10 @@
     </row>
     <row r="240" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B240" s="45" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="C240" s="3" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="D240" s="1" t="n">
         <v>8</v>
@@ -12231,13 +12237,13 @@
       </c>
       <c r="F240" s="34"/>
       <c r="G240" s="34" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="H240" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I240" s="34" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J240" s="42" t="n">
         <f aca="false">J239+D239</f>
@@ -12256,7 +12262,7 @@
         <v>6.75</v>
       </c>
       <c r="N240" s="1" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="O240" s="3" t="n">
         <v>3</v>
@@ -12270,10 +12276,10 @@
     </row>
     <row r="241" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B241" s="45" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="C241" s="3" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="D241" s="1" t="n">
         <v>8</v>
@@ -12283,13 +12289,13 @@
       </c>
       <c r="F241" s="34"/>
       <c r="G241" s="34" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="H241" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I241" s="34" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J241" s="42" t="n">
         <f aca="false">J240+D240</f>
@@ -12308,7 +12314,7 @@
         <v>7</v>
       </c>
       <c r="N241" s="1" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="O241" s="3" t="n">
         <v>3</v>
@@ -12322,10 +12328,10 @@
     </row>
     <row r="242" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B242" s="45" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="C242" s="3" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="D242" s="1" t="n">
         <v>8</v>
@@ -12335,13 +12341,13 @@
       </c>
       <c r="F242" s="34"/>
       <c r="G242" s="34" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="H242" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I242" s="34" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J242" s="42" t="n">
         <f aca="false">J241+D241</f>
@@ -12360,7 +12366,7 @@
         <v>7.25</v>
       </c>
       <c r="N242" s="1" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="O242" s="3" t="n">
         <v>3</v>
@@ -12374,10 +12380,10 @@
     </row>
     <row r="243" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B243" s="45" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="C243" s="3" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="D243" s="1" t="n">
         <v>8</v>
@@ -12387,13 +12393,13 @@
       </c>
       <c r="F243" s="34"/>
       <c r="G243" s="34" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="H243" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I243" s="34" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J243" s="42" t="n">
         <f aca="false">J242+D242</f>
@@ -12412,7 +12418,7 @@
         <v>7.5</v>
       </c>
       <c r="N243" s="1" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="O243" s="3" t="n">
         <v>3</v>
@@ -12426,10 +12432,10 @@
     </row>
     <row r="244" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B244" s="45" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="C244" s="3" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="D244" s="1" t="n">
         <v>8</v>
@@ -12439,13 +12445,13 @@
       </c>
       <c r="F244" s="34"/>
       <c r="G244" s="34" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="H244" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I244" s="34" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J244" s="42" t="n">
         <f aca="false">J243+D243</f>
@@ -12464,7 +12470,7 @@
         <v>7.75</v>
       </c>
       <c r="N244" s="1" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="O244" s="3" t="n">
         <v>3</v>
@@ -12478,10 +12484,10 @@
     </row>
     <row r="245" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B245" s="45" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="C245" s="3" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="D245" s="1" t="n">
         <v>8</v>
@@ -12491,13 +12497,13 @@
       </c>
       <c r="F245" s="34"/>
       <c r="G245" s="34" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="H245" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I245" s="34" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J245" s="42" t="n">
         <f aca="false">J244+D244</f>
@@ -12516,7 +12522,7 @@
         <v>8</v>
       </c>
       <c r="N245" s="1" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="O245" s="3" t="n">
         <v>3</v>
@@ -12530,10 +12536,10 @@
     </row>
     <row r="246" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B246" s="45" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="C246" s="3" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="D246" s="1" t="n">
         <v>16</v>
@@ -12545,13 +12551,13 @@
         <v>116</v>
       </c>
       <c r="G246" s="34" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="H246" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I246" s="34" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J246" s="42" t="n">
         <f aca="false">J245+D245</f>
@@ -12570,7 +12576,7 @@
         <v>8.25</v>
       </c>
       <c r="N246" s="1" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="O246" s="3" t="n">
         <v>1</v>
@@ -12584,10 +12590,10 @@
     </row>
     <row r="247" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B247" s="45" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="C247" s="3" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="D247" s="1" t="n">
         <v>8</v>
@@ -12597,13 +12603,13 @@
       </c>
       <c r="F247" s="34"/>
       <c r="G247" s="34" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="H247" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I247" s="34" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="J247" s="42" t="n">
         <f aca="false">J246+D246</f>
@@ -12622,7 +12628,7 @@
         <v>8.75</v>
       </c>
       <c r="N247" s="1" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="O247" s="3" t="n">
         <v>2</v>
@@ -12726,22 +12732,22 @@
     <row r="6" s="47" customFormat="true" ht="34.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="48"/>
       <c r="C6" s="48" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="D6" s="48" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="E6" s="48" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="F6" s="48" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="G6" s="48" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="H6" s="48" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="I6" s="48"/>
     </row>
@@ -13111,10 +13117,10 @@
     </row>
     <row r="26" s="1" customFormat="true" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="28" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="C26" s="28" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="D26" s="25" t="n">
         <v>16</v>
@@ -13127,10 +13133,10 @@
         <v>1</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="I26" s="26" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="J26" s="26" t="n">
         <f aca="false">DownlinkSpecLTM!J151+DownlinkSpecLTM!D151</f>
@@ -13149,7 +13155,7 @@
         <v>18.5</v>
       </c>
       <c r="N26" s="1" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="O26" s="3" t="n">
         <v>6</v>
@@ -13163,10 +13169,10 @@
     </row>
     <row r="27" s="1" customFormat="true" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="28" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="C27" s="28" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="D27" s="25" t="n">
         <v>32</v>
@@ -13177,10 +13183,10 @@
         <v>1</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="I27" s="26" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="J27" s="26" t="n">
         <f aca="false">J26+D26</f>
@@ -13199,7 +13205,7 @@
         <v>19</v>
       </c>
       <c r="N27" s="1" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="O27" s="3" t="n">
         <v>6</v>
@@ -13213,16 +13219,16 @@
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="46" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="C30" s="46" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="D30" s="46" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="E30" s="46" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="F30" s="46"/>
     </row>

</xml_diff>

<commit_message>
And a few more...
</commit_message>
<xml_diff>
--- a/genSpacecraft/DownlinkSpecFoxPlus-A.xlsx
+++ b/genSpacecraft/DownlinkSpecFoxPlus-A.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1380" uniqueCount="522">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1391" uniqueCount="523">
   <si>
     <t xml:space="preserve">//</t>
   </si>
@@ -1022,7 +1022,7 @@
     <t xml:space="preserve">Modulator Register 0 - Local Oscillator</t>
   </si>
   <si>
-    <t xml:space="preserve">Modulator Reg 1</t>
+    <t xml:space="preserve">Modulator Gain</t>
   </si>
   <si>
     <t xml:space="preserve">ModuGain</t>
@@ -1271,7 +1271,7 @@
     <t xml:space="preserve">pad191</t>
   </si>
   <si>
-    <t xml:space="preserve">Structure:scienceLong_t, file:sciLongDownlink.h</t>
+    <t xml:space="preserve">//Structure:scienceLong_t, file:sciLongDownlink.h</t>
   </si>
   <si>
     <t xml:space="preserve">Data</t>
@@ -1301,7 +1301,10 @@
     <t xml:space="preserve">CAN Queue</t>
   </si>
   <si>
-    <t xml:space="preserve">Structure:science_t, file:sciDownlink.h</t>
+    <t xml:space="preserve">//END</t>
+  </si>
+  <si>
+    <t xml:space="preserve">//Structure:science_t, file:sciDownlink.h</t>
   </si>
   <si>
     <t xml:space="preserve">Sparebits</t>
@@ -1310,7 +1313,7 @@
     <t xml:space="preserve">sparebits</t>
   </si>
   <si>
-    <t xml:space="preserve">Structure:sciWodSpecific_t,file:sciWodSpecificDownlink.h</t>
+    <t xml:space="preserve">//Structure:sciWodSpecific_t,file:sciWodSpecificDownlink.h</t>
   </si>
   <si>
     <t xml:space="preserve">sec</t>
@@ -9806,6 +9809,9 @@
       </c>
     </row>
     <row r="181" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A181" s="38" t="s">
+        <v>0</v>
+      </c>
       <c r="B181" s="27" t="s">
         <v>417</v>
       </c>
@@ -9859,6 +9865,9 @@
       </c>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A182" s="38" t="s">
+        <v>0</v>
+      </c>
       <c r="B182" s="27" t="s">
         <v>420</v>
       </c>
@@ -9911,6 +9920,9 @@
       </c>
     </row>
     <row r="183" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A183" s="38" t="s">
+        <v>0</v>
+      </c>
       <c r="B183" s="27" t="s">
         <v>422</v>
       </c>
@@ -9962,7 +9974,7 @@
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="1" t="s">
-        <v>59</v>
+        <v>426</v>
       </c>
       <c r="I184" s="1" t="s">
         <v>241</v>
@@ -9985,6 +9997,9 @@
       </c>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A185" s="38" t="s">
+        <v>0</v>
+      </c>
       <c r="B185" s="27"/>
       <c r="J185" s="26"/>
       <c r="K185" s="26"/>
@@ -9993,7 +10008,7 @@
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="40" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="B186" s="10"/>
       <c r="C186" s="39"/>
@@ -10058,6 +10073,9 @@
       </c>
     </row>
     <row r="188" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A188" s="38" t="s">
+        <v>0</v>
+      </c>
       <c r="B188" s="27" t="s">
         <v>417</v>
       </c>
@@ -10111,11 +10129,14 @@
       </c>
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A189" s="38" t="s">
+        <v>0</v>
+      </c>
       <c r="B189" s="27" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="C189" s="20" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="D189" s="20" t="n">
         <v>7</v>
@@ -10163,6 +10184,9 @@
       </c>
     </row>
     <row r="190" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A190" s="38" t="s">
+        <v>0</v>
+      </c>
       <c r="B190" s="27" t="s">
         <v>422</v>
       </c>
@@ -10214,7 +10238,7 @@
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A191" s="1" t="s">
-        <v>59</v>
+        <v>426</v>
       </c>
       <c r="I191" s="1" t="s">
         <v>241</v>
@@ -10238,7 +10262,7 @@
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A195" s="40" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="B195" s="10"/>
       <c r="C195" s="39"/>
@@ -10303,6 +10327,9 @@
       </c>
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A197" s="1" t="s">
+        <v>0</v>
+      </c>
       <c r="B197" s="27" t="s">
         <v>404</v>
       </c>
@@ -10320,7 +10347,7 @@
         <v>1</v>
       </c>
       <c r="H197" s="37" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="I197" s="26" t="s">
         <v>406</v>
@@ -10355,6 +10382,9 @@
       </c>
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A198" s="1" t="s">
+        <v>0</v>
+      </c>
       <c r="B198" s="27" t="s">
         <v>407</v>
       </c>
@@ -10409,8 +10439,11 @@
       </c>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A199" s="1" t="s">
+        <v>0</v>
+      </c>
       <c r="B199" s="27" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="C199" s="28" t="s">
         <v>412</v>
@@ -10427,7 +10460,7 @@
         <v>27</v>
       </c>
       <c r="I199" s="26" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="J199" s="4" t="n">
         <f aca="false">J198+D198</f>
@@ -10459,11 +10492,14 @@
       </c>
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A200" s="1" t="s">
+        <v>0</v>
+      </c>
       <c r="B200" s="27" t="s">
         <v>28</v>
       </c>
       <c r="C200" s="28" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="D200" s="25" t="n">
         <v>8</v>
@@ -10510,7 +10546,7 @@
     </row>
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A201" s="1" t="s">
-        <v>59</v>
+        <v>426</v>
       </c>
       <c r="I201" s="1" t="s">
         <v>241</v>
@@ -10546,7 +10582,7 @@
     </row>
     <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A203" s="40" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
     </row>
     <row r="204" s="13" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10603,8 +10639,9 @@
       </c>
     </row>
     <row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A205" s="38"/>
       <c r="B205" s="41" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="C205" s="34" t="s">
         <v>404</v>
@@ -10620,10 +10657,10 @@
         <v>379</v>
       </c>
       <c r="H205" s="34" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="I205" s="34" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="J205" s="42" t="n">
         <v>0</v>
@@ -10641,7 +10678,7 @@
         <v>0</v>
       </c>
       <c r="N205" s="1" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="O205" s="3" t="n">
         <v>1</v>
@@ -10654,11 +10691,12 @@
       </c>
     </row>
     <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A206" s="38"/>
       <c r="B206" s="41" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="C206" s="34" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="D206" s="34" t="n">
         <v>32</v>
@@ -10671,10 +10709,10 @@
         <v>379</v>
       </c>
       <c r="H206" s="34" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="I206" s="34" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="J206" s="42" t="n">
         <f aca="false">J205+D205</f>
@@ -10693,7 +10731,7 @@
         <v>1</v>
       </c>
       <c r="N206" s="1" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="O206" s="3" t="n">
         <v>1</v>
@@ -10707,7 +10745,7 @@
     </row>
     <row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A207" s="1" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="B207" s="41"/>
       <c r="C207" s="34"/>
@@ -10724,10 +10762,10 @@
     </row>
     <row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B208" s="41" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="C208" s="34" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="D208" s="34" t="n">
         <v>1</v>
@@ -10737,13 +10775,13 @@
       </c>
       <c r="F208" s="34"/>
       <c r="G208" s="34" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="H208" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I208" s="34" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J208" s="42" t="n">
         <f aca="false">J206+D206</f>
@@ -10762,7 +10800,7 @@
         <v>2</v>
       </c>
       <c r="N208" s="1" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="O208" s="3" t="n">
         <v>1</v>
@@ -10776,10 +10814,10 @@
     </row>
     <row r="209" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B209" s="41" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C209" s="34" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D209" s="34" t="n">
         <v>5</v>
@@ -10793,7 +10831,7 @@
       </c>
       <c r="H209" s="34"/>
       <c r="I209" s="34" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="J209" s="42" t="n">
         <f aca="false">J208+D208</f>
@@ -10812,7 +10850,7 @@
         <v>2.03125</v>
       </c>
       <c r="N209" s="1" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="O209" s="3" t="n">
         <v>1</v>
@@ -10826,10 +10864,10 @@
     </row>
     <row r="210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B210" s="41" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="C210" s="34" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="D210" s="34" t="n">
         <v>4</v>
@@ -10845,7 +10883,7 @@
         <v>27</v>
       </c>
       <c r="I210" s="34" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J210" s="42" t="n">
         <f aca="false">J209+D209</f>
@@ -10864,7 +10902,7 @@
         <v>2.1875</v>
       </c>
       <c r="N210" s="1" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="O210" s="3" t="n">
         <v>1</v>
@@ -10878,10 +10916,10 @@
     </row>
     <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B211" s="41" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="C211" s="34" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="D211" s="34" t="n">
         <v>5</v>
@@ -10897,7 +10935,7 @@
         <v>27</v>
       </c>
       <c r="I211" s="34" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J211" s="42" t="n">
         <f aca="false">J210+D210</f>
@@ -10916,7 +10954,7 @@
         <v>2.3125</v>
       </c>
       <c r="N211" s="1" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="O211" s="3" t="n">
         <v>1</v>
@@ -10930,10 +10968,10 @@
     </row>
     <row r="212" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B212" s="41" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C212" s="34" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="D212" s="34" t="n">
         <v>6</v>
@@ -10949,7 +10987,7 @@
         <v>27</v>
       </c>
       <c r="I212" s="34" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J212" s="42" t="n">
         <f aca="false">J211+D211</f>
@@ -10968,7 +11006,7 @@
         <v>2.46875</v>
       </c>
       <c r="N212" s="1" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="O212" s="3" t="n">
         <v>1</v>
@@ -10982,10 +11020,10 @@
     </row>
     <row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B213" s="41" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C213" s="34" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="D213" s="34" t="n">
         <v>6</v>
@@ -11001,7 +11039,7 @@
         <v>27</v>
       </c>
       <c r="I213" s="34" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J213" s="42" t="n">
         <f aca="false">J212+D212</f>
@@ -11020,7 +11058,7 @@
         <v>2.65625</v>
       </c>
       <c r="N213" s="1" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="O213" s="3" t="n">
         <v>1</v>
@@ -11034,10 +11072,10 @@
     </row>
     <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B214" s="41" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C214" s="34" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D214" s="34" t="n">
         <v>5</v>
@@ -11053,7 +11091,7 @@
         <v>27</v>
       </c>
       <c r="I214" s="34" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J214" s="42" t="n">
         <f aca="false">J213+D213</f>
@@ -11072,7 +11110,7 @@
         <v>2.84375</v>
       </c>
       <c r="N214" s="1" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="O214" s="3" t="n">
         <v>1</v>
@@ -11086,7 +11124,7 @@
     </row>
     <row r="215" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A215" s="1" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="B215" s="41"/>
       <c r="C215" s="34"/>
@@ -11103,10 +11141,10 @@
     </row>
     <row r="216" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B216" s="41" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="C216" s="34" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="D216" s="34" t="n">
         <v>8</v>
@@ -11122,7 +11160,7 @@
         <v>71</v>
       </c>
       <c r="I216" s="34" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J216" s="42" t="n">
         <f aca="false">J214+D214</f>
@@ -11141,7 +11179,7 @@
         <v>3</v>
       </c>
       <c r="N216" s="1" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="O216" s="3" t="n">
         <v>1</v>
@@ -11155,10 +11193,10 @@
     </row>
     <row r="217" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B217" s="41" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="C217" s="34" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="D217" s="34" t="n">
         <v>8</v>
@@ -11174,7 +11212,7 @@
         <v>71</v>
       </c>
       <c r="I217" s="34" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J217" s="42" t="n">
         <f aca="false">J216+D216</f>
@@ -11193,7 +11231,7 @@
         <v>3.25</v>
       </c>
       <c r="N217" s="1" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="O217" s="3" t="n">
         <v>1</v>
@@ -11207,10 +11245,10 @@
     </row>
     <row r="218" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B218" s="41" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="C218" s="34" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="D218" s="34" t="n">
         <v>8</v>
@@ -11226,7 +11264,7 @@
         <v>27</v>
       </c>
       <c r="I218" s="34" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J218" s="42" t="n">
         <f aca="false">J217+D217</f>
@@ -11259,10 +11297,10 @@
     </row>
     <row r="219" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B219" s="41" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="C219" s="34" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="D219" s="34" t="n">
         <v>8</v>
@@ -11272,13 +11310,13 @@
       </c>
       <c r="F219" s="34"/>
       <c r="G219" s="34" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="H219" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I219" s="34" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J219" s="42" t="n">
         <f aca="false">J218+D218</f>
@@ -11297,7 +11335,7 @@
         <v>3.75</v>
       </c>
       <c r="N219" s="1" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="O219" s="3" t="n">
         <v>2</v>
@@ -11341,7 +11379,7 @@
     </row>
     <row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A221" s="40" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="F221" s="34"/>
       <c r="G221" s="34"/>
@@ -11425,10 +11463,10 @@
     </row>
     <row r="224" s="45" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B224" s="19" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="C224" s="43" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="D224" s="1" t="n">
         <v>5</v>
@@ -11444,7 +11482,7 @@
         <v>27</v>
       </c>
       <c r="I224" s="34" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J224" s="42" t="n">
         <f aca="false">J220</f>
@@ -11477,10 +11515,10 @@
     </row>
     <row r="225" s="45" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B225" s="19" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="C225" s="43" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="D225" s="1" t="n">
         <v>1</v>
@@ -11490,13 +11528,13 @@
       </c>
       <c r="F225" s="44"/>
       <c r="G225" s="34" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="H225" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I225" s="34" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J225" s="42" t="n">
         <f aca="false">J224+D224</f>
@@ -11515,7 +11553,7 @@
         <v>4.15625</v>
       </c>
       <c r="N225" s="1" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="O225" s="3" t="n">
         <v>1</v>
@@ -11529,10 +11567,10 @@
     </row>
     <row r="226" s="45" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B226" s="19" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="C226" s="43" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="D226" s="1" t="n">
         <v>1</v>
@@ -11542,13 +11580,13 @@
       </c>
       <c r="F226" s="44"/>
       <c r="G226" s="34" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="H226" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I226" s="34" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J226" s="42" t="n">
         <f aca="false">J225+D225</f>
@@ -11567,7 +11605,7 @@
         <v>4.1875</v>
       </c>
       <c r="N226" s="1" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="O226" s="3" t="n">
         <v>2</v>
@@ -11581,10 +11619,10 @@
     </row>
     <row r="227" s="45" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B227" s="19" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="C227" s="43" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="D227" s="1" t="n">
         <v>3</v>
@@ -11600,7 +11638,7 @@
         <v>27</v>
       </c>
       <c r="I227" s="34" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J227" s="42" t="n">
         <f aca="false">J226+D226</f>
@@ -11619,7 +11657,7 @@
         <v>4.21875</v>
       </c>
       <c r="N227" s="1" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="O227" s="3" t="n">
         <v>2</v>
@@ -11633,10 +11671,10 @@
     </row>
     <row r="228" s="45" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B228" s="19" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="C228" s="43" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="D228" s="1" t="n">
         <v>4</v>
@@ -11646,13 +11684,13 @@
       </c>
       <c r="F228" s="44"/>
       <c r="G228" s="34" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="H228" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I228" s="34" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J228" s="42" t="n">
         <f aca="false">J227+D227</f>
@@ -11671,7 +11709,7 @@
         <v>4.3125</v>
       </c>
       <c r="N228" s="1" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="O228" s="3" t="n">
         <v>2</v>
@@ -11685,10 +11723,10 @@
     </row>
     <row r="229" s="45" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B229" s="19" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="C229" s="43" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="D229" s="1" t="n">
         <v>4</v>
@@ -11698,13 +11736,13 @@
       </c>
       <c r="F229" s="44"/>
       <c r="G229" s="34" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="H229" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I229" s="34" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J229" s="42" t="n">
         <f aca="false">J228+D228</f>
@@ -11723,7 +11761,7 @@
         <v>4.4375</v>
       </c>
       <c r="N229" s="1" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="O229" s="3" t="n">
         <v>2</v>
@@ -11737,10 +11775,10 @@
     </row>
     <row r="230" s="45" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B230" s="19" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="C230" s="43" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="D230" s="1" t="n">
         <v>5</v>
@@ -11750,13 +11788,13 @@
       </c>
       <c r="F230" s="44"/>
       <c r="G230" s="34" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="H230" s="34" t="s">
         <v>27</v>
       </c>
       <c r="I230" s="34" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J230" s="42" t="n">
         <f aca="false">J229+D229</f>
@@ -11775,7 +11813,7 @@
         <v>4.5625</v>
       </c>
       <c r="N230" s="1" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="O230" s="3" t="n">
         <v>2</v>
@@ -11789,10 +11827,10 @@
     </row>
     <row r="231" s="45" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B231" s="19" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="C231" s="43" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="D231" s="1" t="n">
         <v>9</v>
@@ -11808,7 +11846,7 @@
         <v>27</v>
       </c>
       <c r="I231" s="34" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J231" s="42" t="n">
         <f aca="false">J230+D230</f>
@@ -11827,7 +11865,7 @@
         <v>4.71875</v>
       </c>
       <c r="N231" s="1" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="O231" s="3" t="n">
         <v>2</v>
@@ -11860,10 +11898,10 @@
     </row>
     <row r="233" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B233" s="45" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="C233" s="3" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="D233" s="1" t="n">
         <v>8</v>
@@ -11879,7 +11917,7 @@
         <v>27</v>
       </c>
       <c r="I233" s="34" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J233" s="42" t="n">
         <f aca="false">J231+D231</f>
@@ -11898,7 +11936,7 @@
         <v>5</v>
       </c>
       <c r="N233" s="1" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="O233" s="3" t="n">
         <v>3</v>
@@ -11912,10 +11950,10 @@
     </row>
     <row r="234" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B234" s="45" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="C234" s="3" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="D234" s="1" t="n">
         <v>8</v>
@@ -11931,7 +11969,7 @@
         <v>27</v>
       </c>
       <c r="I234" s="34" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J234" s="42" t="n">
         <f aca="false">J233+D233</f>
@@ -11950,7 +11988,7 @@
         <v>5.25</v>
       </c>
       <c r="N234" s="1" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="O234" s="3" t="n">
         <v>3</v>
@@ -11964,10 +12002,10 @@
     </row>
     <row r="235" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B235" s="45" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="C235" s="3" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="D235" s="1" t="n">
         <v>8</v>
@@ -11983,7 +12021,7 @@
         <v>27</v>
       </c>
       <c r="I235" s="34" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J235" s="42" t="n">
         <f aca="false">J234+D234</f>
@@ -12002,7 +12040,7 @@
         <v>5.5</v>
       </c>
       <c r="N235" s="1" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="O235" s="3" t="n">
         <v>3</v>
@@ -12016,10 +12054,10 @@
     </row>
     <row r="236" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B236" s="45" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="C236" s="3" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="D236" s="1" t="n">
         <v>8</v>
@@ -12035,7 +12073,7 @@
         <v>27</v>
       </c>
       <c r="I236" s="34" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J236" s="42" t="n">
         <f aca="false">J235+D235</f>
@@ -12054,7 +12092,7 @@
         <v>5.75</v>
       </c>
       <c r="N236" s="1" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="O236" s="3" t="n">
         <v>3</v>
@@ -12068,10 +12106,10 @@
     </row>
     <row r="237" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B237" s="45" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="C237" s="3" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="D237" s="1" t="n">
         <v>8</v>
@@ -12087,7 +12125,7 @@
         <v>27</v>
       </c>
       <c r="I237" s="34" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J237" s="42" t="n">
         <f aca="false">J236+D236</f>
@@ -12106,7 +12144,7 @@
         <v>6</v>
       </c>
       <c r="N237" s="1" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="O237" s="3" t="n">
         <v>3</v>
@@ -12120,10 +12158,10 @@
     </row>
     <row r="238" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B238" s="45" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="C238" s="3" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="D238" s="1" t="n">
         <v>8</v>
@@ -12139,7 +12177,7 @@
         <v>27</v>
       </c>
       <c r="I238" s="34" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J238" s="42" t="n">
         <f aca="false">J237+D237</f>
@@ -12158,7 +12196,7 @@
         <v>6.25</v>
       </c>
       <c r="N238" s="1" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="O238" s="3" t="n">
         <v>3</v>
@@ -12172,10 +12210,10 @@
     </row>
     <row r="239" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B239" s="45" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="C239" s="3" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="D239" s="1" t="n">
         <v>8</v>
@@ -12191,7 +12229,7 @@
         <v>27</v>
       </c>
       <c r="I239" s="34" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J239" s="42" t="n">
         <f aca="false">J238+D238</f>
@@ -12210,7 +12248,7 @@
         <v>6.5</v>
       </c>
       <c r="N239" s="1" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="O239" s="3" t="n">
         <v>3</v>
@@ -12224,10 +12262,10 @@
     </row>
     <row r="240" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B240" s="45" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="C240" s="3" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="D240" s="1" t="n">
         <v>8</v>
@@ -12243,7 +12281,7 @@
         <v>27</v>
       </c>
       <c r="I240" s="34" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J240" s="42" t="n">
         <f aca="false">J239+D239</f>
@@ -12262,7 +12300,7 @@
         <v>6.75</v>
       </c>
       <c r="N240" s="1" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="O240" s="3" t="n">
         <v>3</v>
@@ -12276,10 +12314,10 @@
     </row>
     <row r="241" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B241" s="45" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="C241" s="3" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="D241" s="1" t="n">
         <v>8</v>
@@ -12295,7 +12333,7 @@
         <v>27</v>
       </c>
       <c r="I241" s="34" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J241" s="42" t="n">
         <f aca="false">J240+D240</f>
@@ -12314,7 +12352,7 @@
         <v>7</v>
       </c>
       <c r="N241" s="1" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="O241" s="3" t="n">
         <v>3</v>
@@ -12328,10 +12366,10 @@
     </row>
     <row r="242" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B242" s="45" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C242" s="3" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="D242" s="1" t="n">
         <v>8</v>
@@ -12347,7 +12385,7 @@
         <v>27</v>
       </c>
       <c r="I242" s="34" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J242" s="42" t="n">
         <f aca="false">J241+D241</f>
@@ -12366,7 +12404,7 @@
         <v>7.25</v>
       </c>
       <c r="N242" s="1" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="O242" s="3" t="n">
         <v>3</v>
@@ -12380,10 +12418,10 @@
     </row>
     <row r="243" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B243" s="45" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="C243" s="3" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="D243" s="1" t="n">
         <v>8</v>
@@ -12399,7 +12437,7 @@
         <v>27</v>
       </c>
       <c r="I243" s="34" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J243" s="42" t="n">
         <f aca="false">J242+D242</f>
@@ -12418,7 +12456,7 @@
         <v>7.5</v>
       </c>
       <c r="N243" s="1" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="O243" s="3" t="n">
         <v>3</v>
@@ -12432,10 +12470,10 @@
     </row>
     <row r="244" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B244" s="45" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="C244" s="3" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="D244" s="1" t="n">
         <v>8</v>
@@ -12451,7 +12489,7 @@
         <v>27</v>
       </c>
       <c r="I244" s="34" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J244" s="42" t="n">
         <f aca="false">J243+D243</f>
@@ -12470,7 +12508,7 @@
         <v>7.75</v>
       </c>
       <c r="N244" s="1" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="O244" s="3" t="n">
         <v>3</v>
@@ -12484,10 +12522,10 @@
     </row>
     <row r="245" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B245" s="45" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="C245" s="3" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="D245" s="1" t="n">
         <v>8</v>
@@ -12503,7 +12541,7 @@
         <v>27</v>
       </c>
       <c r="I245" s="34" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J245" s="42" t="n">
         <f aca="false">J244+D244</f>
@@ -12522,7 +12560,7 @@
         <v>8</v>
       </c>
       <c r="N245" s="1" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="O245" s="3" t="n">
         <v>3</v>
@@ -12536,10 +12574,10 @@
     </row>
     <row r="246" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B246" s="45" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="C246" s="3" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="D246" s="1" t="n">
         <v>16</v>
@@ -12557,7 +12595,7 @@
         <v>27</v>
       </c>
       <c r="I246" s="34" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J246" s="42" t="n">
         <f aca="false">J245+D245</f>
@@ -12576,7 +12614,7 @@
         <v>8.25</v>
       </c>
       <c r="N246" s="1" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="O246" s="3" t="n">
         <v>1</v>
@@ -12590,10 +12628,10 @@
     </row>
     <row r="247" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B247" s="45" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="C247" s="3" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="D247" s="1" t="n">
         <v>8</v>
@@ -12609,7 +12647,7 @@
         <v>27</v>
       </c>
       <c r="I247" s="34" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="J247" s="42" t="n">
         <f aca="false">J246+D246</f>
@@ -12628,7 +12666,7 @@
         <v>8.75</v>
       </c>
       <c r="N247" s="1" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="O247" s="3" t="n">
         <v>2</v>
@@ -12698,11 +12736,9 @@
     <mergeCell ref="B87:I87"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A179" r:id="rId1" display="Structure:scienceLong_t, file:sciLongDownlink.h"/>
-    <hyperlink ref="A186" r:id="rId2" display="Structure:science_t, file:sciDownlink.h"/>
-    <hyperlink ref="A195" r:id="rId3" display="Structure:sciWodSpecific_t,file:sciWodSpecificDownlink.h"/>
-    <hyperlink ref="A203" r:id="rId4" display="Structure:infrequentDownlink_t,file:infrequentDownlink.h"/>
-    <hyperlink ref="A221" r:id="rId5" display="Structure:legacyErrors_t,file:legacyErrorsDownlink.h"/>
+    <hyperlink ref="A186" r:id="rId1" display="//Structure:science_t, file:sciDownlink.h"/>
+    <hyperlink ref="A203" r:id="rId2" display="Structure:infrequentDownlink_t,file:infrequentDownlink.h"/>
+    <hyperlink ref="A221" r:id="rId3" display="Structure:legacyErrors_t,file:legacyErrorsDownlink.h"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
@@ -12732,22 +12768,22 @@
     <row r="6" s="47" customFormat="true" ht="34.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="48"/>
       <c r="C6" s="48" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="D6" s="48" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E6" s="48" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="F6" s="48" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="G6" s="48" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="H6" s="48" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="I6" s="48"/>
     </row>
@@ -13117,10 +13153,10 @@
     </row>
     <row r="26" s="1" customFormat="true" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="28" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="C26" s="28" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="D26" s="25" t="n">
         <v>16</v>
@@ -13155,7 +13191,7 @@
         <v>18.5</v>
       </c>
       <c r="N26" s="1" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="O26" s="3" t="n">
         <v>6</v>
@@ -13169,10 +13205,10 @@
     </row>
     <row r="27" s="1" customFormat="true" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="28" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="C27" s="28" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="D27" s="25" t="n">
         <v>32</v>
@@ -13205,7 +13241,7 @@
         <v>19</v>
       </c>
       <c r="N27" s="1" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="O27" s="3" t="n">
         <v>6</v>
@@ -13219,16 +13255,16 @@
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="46" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="C30" s="46" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="D30" s="46" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="E30" s="46" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="F30" s="46"/>
     </row>

</xml_diff>